<commit_message>
Corregido exe y rutas
</commit_message>
<xml_diff>
--- a/clean_data/model_IG.xlsx
+++ b/clean_data/model_IG.xlsx
@@ -447,10 +447,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B2" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C2" t="n">
         <v>6</v>
@@ -458,10 +458,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B3" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C3" t="n">
         <v>6</v>
@@ -469,10 +469,10 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B4" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C4" t="n">
         <v>5</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B5" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C5" t="n">
         <v>3</v>
@@ -491,10 +491,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B6" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C6" t="n">
         <v>5</v>
@@ -502,10 +502,10 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B7" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C7" t="n">
         <v>6</v>
@@ -516,7 +516,7 @@
         <v>3.64</v>
       </c>
       <c r="B8" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C8" t="n">
         <v>8</v>
@@ -524,10 +524,10 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B9" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C9" t="n">
         <v>5</v>
@@ -535,10 +535,10 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B10" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C10" t="n">
         <v>6</v>
@@ -546,10 +546,10 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B11" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C11" t="n">
         <v>5</v>
@@ -557,10 +557,10 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B12" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C12" t="n">
         <v>7</v>
@@ -568,10 +568,10 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B13" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C13" t="n">
         <v>5</v>
@@ -579,10 +579,10 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B14" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C14" t="n">
         <v>6</v>
@@ -590,10 +590,10 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B15" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -601,10 +601,10 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B16" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C16" t="n">
         <v>6</v>
@@ -612,10 +612,10 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B17" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C17" t="n">
         <v>3</v>
@@ -623,10 +623,10 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B18" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C18" t="n">
         <v>4</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B19" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C19" t="n">
         <v>6</v>
@@ -645,10 +645,10 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B20" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C20" t="n">
         <v>6</v>
@@ -656,10 +656,10 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B21" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C21" t="n">
         <v>5</v>
@@ -670,7 +670,7 @@
         <v>3.64</v>
       </c>
       <c r="B22" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C22" t="n">
         <v>8</v>
@@ -678,10 +678,10 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B23" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C23" t="n">
         <v>5</v>
@@ -689,10 +689,10 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B24" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C24" t="n">
         <v>6</v>
@@ -700,10 +700,10 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B25" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C25" t="n">
         <v>6</v>
@@ -711,10 +711,10 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B26" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C26" t="n">
         <v>5</v>
@@ -722,10 +722,10 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B27" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C27" t="n">
         <v>5</v>
@@ -733,10 +733,10 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B28" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C28" t="n">
         <v>6</v>
@@ -744,10 +744,10 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B29" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C29" t="n">
         <v>6</v>
@@ -755,10 +755,10 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B30" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C30" t="n">
         <v>5</v>
@@ -766,10 +766,10 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B31" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C31" t="n">
         <v>7</v>
@@ -777,10 +777,10 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B32" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C32" t="n">
         <v>4</v>
@@ -788,10 +788,10 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B33" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C33" t="n">
         <v>7</v>
@@ -799,10 +799,10 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B34" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C34" t="n">
         <v>6</v>
@@ -810,10 +810,10 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B35" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C35" t="n">
         <v>7</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B36" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C36" t="n">
         <v>7</v>
@@ -832,10 +832,10 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B37" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C37" t="n">
         <v>6</v>
@@ -843,10 +843,10 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B38" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C38" t="n">
         <v>7</v>
@@ -854,10 +854,10 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B39" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C39" t="n">
         <v>6</v>
@@ -865,10 +865,10 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B40" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C40" t="n">
         <v>6</v>
@@ -876,10 +876,10 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B41" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C41" t="n">
         <v>5</v>
@@ -887,10 +887,10 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B42" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C42" t="n">
         <v>6</v>
@@ -898,10 +898,10 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4.84</v>
+        <v>4.35</v>
       </c>
       <c r="B43" t="n">
-        <v>10.51</v>
+        <v>12.66</v>
       </c>
       <c r="C43" t="n">
         <v>11</v>
@@ -909,10 +909,10 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B44" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C44" t="n">
         <v>5</v>
@@ -920,10 +920,10 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B45" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C45" t="n">
         <v>6</v>
@@ -931,10 +931,10 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B46" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C46" t="n">
         <v>5</v>
@@ -942,10 +942,10 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B47" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C47" t="n">
         <v>7</v>
@@ -953,10 +953,10 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B48" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C48" t="n">
         <v>5</v>
@@ -964,10 +964,10 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B49" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C49" t="n">
         <v>7</v>
@@ -975,10 +975,10 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B50" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C50" t="n">
         <v>5</v>
@@ -986,10 +986,10 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B51" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C51" t="n">
         <v>5</v>
@@ -997,10 +997,10 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B52" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C52" t="n">
         <v>6</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B53" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C53" t="n">
         <v>4</v>
@@ -1019,10 +1019,10 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B54" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C54" t="n">
         <v>6</v>
@@ -1030,10 +1030,10 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B55" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C55" t="n">
         <v>5</v>
@@ -1041,10 +1041,10 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B56" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C56" t="n">
         <v>7</v>
@@ -1052,10 +1052,10 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>4.04</v>
+        <v>3.88</v>
       </c>
       <c r="B57" t="n">
-        <v>8.69</v>
+        <v>10.93</v>
       </c>
       <c r="C57" t="n">
         <v>9</v>
@@ -1063,10 +1063,10 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B58" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C58" t="n">
         <v>6</v>
@@ -1074,10 +1074,10 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B59" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C59" t="n">
         <v>5</v>
@@ -1085,10 +1085,10 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B60" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C60" t="n">
         <v>4</v>
@@ -1096,10 +1096,10 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B61" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C61" t="n">
         <v>7</v>
@@ -1107,10 +1107,10 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.13</v>
       </c>
       <c r="B62" t="n">
-        <v>1.09</v>
+        <v>2.32</v>
       </c>
       <c r="C62" t="n">
         <v>1</v>
@@ -1118,10 +1118,10 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B63" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C63" t="n">
         <v>6</v>
@@ -1129,10 +1129,10 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B64" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C64" t="n">
         <v>4</v>
@@ -1140,10 +1140,10 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B65" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C65" t="n">
         <v>5</v>
@@ -1151,10 +1151,10 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B66" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C66" t="n">
         <v>5</v>
@@ -1162,10 +1162,10 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B67" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C67" t="n">
         <v>4</v>
@@ -1173,10 +1173,10 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B68" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C68" t="n">
         <v>5</v>
@@ -1184,10 +1184,10 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B69" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C69" t="n">
         <v>5</v>
@@ -1198,7 +1198,7 @@
         <v>3.64</v>
       </c>
       <c r="B70" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C70" t="n">
         <v>8</v>
@@ -1206,10 +1206,10 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B71" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C71" t="n">
         <v>6</v>
@@ -1217,10 +1217,10 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B72" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C72" t="n">
         <v>6</v>
@@ -1228,10 +1228,10 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B73" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C73" t="n">
         <v>6</v>
@@ -1239,10 +1239,10 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B74" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C74" t="n">
         <v>4</v>
@@ -1250,10 +1250,10 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B75" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C75" t="n">
         <v>3</v>
@@ -1261,10 +1261,10 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B76" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C76" t="n">
         <v>4</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B77" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C77" t="n">
         <v>5</v>
@@ -1283,10 +1283,10 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B78" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C78" t="n">
         <v>5</v>
@@ -1294,10 +1294,10 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B79" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C79" t="n">
         <v>3</v>
@@ -1305,10 +1305,10 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B80" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C80" t="n">
         <v>6</v>
@@ -1316,10 +1316,10 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B81" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C81" t="n">
         <v>4</v>
@@ -1327,10 +1327,10 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B82" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C82" t="n">
         <v>6</v>
@@ -1338,10 +1338,10 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B83" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C83" t="n">
         <v>5</v>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B84" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C84" t="n">
         <v>3</v>
@@ -1360,10 +1360,10 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B85" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C85" t="n">
         <v>3</v>
@@ -1371,10 +1371,10 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B86" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C86" t="n">
         <v>6</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B87" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C87" t="n">
         <v>6</v>
@@ -1393,10 +1393,10 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B88" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C88" t="n">
         <v>5</v>
@@ -1404,10 +1404,10 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B89" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C89" t="n">
         <v>6</v>
@@ -1415,10 +1415,10 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B90" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C90" t="n">
         <v>7</v>
@@ -1426,10 +1426,10 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B91" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C91" t="n">
         <v>5</v>
@@ -1437,10 +1437,10 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B92" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C92" t="n">
         <v>4</v>
@@ -1448,10 +1448,10 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B93" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C93" t="n">
         <v>5</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B94" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C94" t="n">
         <v>6</v>
@@ -1470,10 +1470,10 @@
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B95" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C95" t="n">
         <v>5</v>
@@ -1481,10 +1481,10 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B96" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C96" t="n">
         <v>6</v>
@@ -1492,10 +1492,10 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B97" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C97" t="n">
         <v>5</v>
@@ -1503,10 +1503,10 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B98" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C98" t="n">
         <v>6</v>
@@ -1514,10 +1514,10 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B99" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C99" t="n">
         <v>3</v>
@@ -1525,10 +1525,10 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B100" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C100" t="n">
         <v>6</v>
@@ -1536,10 +1536,10 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B101" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C101" t="n">
         <v>7</v>
@@ -1547,10 +1547,10 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B102" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C102" t="n">
         <v>4</v>
@@ -1558,10 +1558,10 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B103" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C103" t="n">
         <v>5</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B104" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C104" t="n">
         <v>6</v>
@@ -1580,10 +1580,10 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B105" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C105" t="n">
         <v>5</v>
@@ -1591,10 +1591,10 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B106" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C106" t="n">
         <v>6</v>
@@ -1602,10 +1602,10 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B107" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C107" t="n">
         <v>5</v>
@@ -1613,10 +1613,10 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B108" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C108" t="n">
         <v>5</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B109" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C109" t="n">
         <v>6</v>
@@ -1635,10 +1635,10 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B110" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C110" t="n">
         <v>7</v>
@@ -1646,10 +1646,10 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B111" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C111" t="n">
         <v>5</v>
@@ -1657,10 +1657,10 @@
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B112" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C112" t="n">
         <v>5</v>
@@ -1668,10 +1668,10 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B113" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C113" t="n">
         <v>4</v>
@@ -1679,10 +1679,10 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B114" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C114" t="n">
         <v>6</v>
@@ -1690,10 +1690,10 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B115" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C115" t="n">
         <v>6</v>
@@ -1701,10 +1701,10 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B116" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C116" t="n">
         <v>5</v>
@@ -1712,10 +1712,10 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B117" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C117" t="n">
         <v>5</v>
@@ -1723,10 +1723,10 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B118" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C118" t="n">
         <v>7</v>
@@ -1734,10 +1734,10 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B119" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C119" t="n">
         <v>5</v>
@@ -1745,10 +1745,10 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B120" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C120" t="n">
         <v>4</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B121" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C121" t="n">
         <v>5</v>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B122" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C122" t="n">
         <v>5</v>
@@ -1778,10 +1778,10 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B123" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C123" t="n">
         <v>6</v>
@@ -1789,10 +1789,10 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B124" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C124" t="n">
         <v>5</v>
@@ -1800,10 +1800,10 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B125" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C125" t="n">
         <v>4</v>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B126" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C126" t="n">
         <v>6</v>
@@ -1822,10 +1822,10 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B127" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C127" t="n">
         <v>6</v>
@@ -1833,10 +1833,10 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B128" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C128" t="n">
         <v>6</v>
@@ -1844,10 +1844,10 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B129" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C129" t="n">
         <v>4</v>
@@ -1855,10 +1855,10 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B130" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C130" t="n">
         <v>4</v>
@@ -1866,10 +1866,10 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B131" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C131" t="n">
         <v>7</v>
@@ -1877,10 +1877,10 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B132" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C132" t="n">
         <v>3</v>
@@ -1888,10 +1888,10 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B133" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C133" t="n">
         <v>6</v>
@@ -1902,7 +1902,7 @@
         <v>3.64</v>
       </c>
       <c r="B134" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C134" t="n">
         <v>8</v>
@@ -1910,10 +1910,10 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B135" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C135" t="n">
         <v>5</v>
@@ -1921,10 +1921,10 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B136" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C136" t="n">
         <v>5</v>
@@ -1932,10 +1932,10 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B137" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C137" t="n">
         <v>4</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B138" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C138" t="n">
         <v>3</v>
@@ -1954,10 +1954,10 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B139" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C139" t="n">
         <v>6</v>
@@ -1965,10 +1965,10 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B140" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C140" t="n">
         <v>5</v>
@@ -1976,10 +1976,10 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B141" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C141" t="n">
         <v>6</v>
@@ -1987,10 +1987,10 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B142" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C142" t="n">
         <v>5</v>
@@ -1998,10 +1998,10 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>4.45</v>
+        <v>4.12</v>
       </c>
       <c r="B143" t="n">
-        <v>9.619999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="C143" t="n">
         <v>10</v>
@@ -2012,7 +2012,7 @@
         <v>3.64</v>
       </c>
       <c r="B144" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C144" t="n">
         <v>8</v>
@@ -2020,10 +2020,10 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B145" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C145" t="n">
         <v>6</v>
@@ -2031,10 +2031,10 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B146" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C146" t="n">
         <v>6</v>
@@ -2042,10 +2042,10 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B147" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C147" t="n">
         <v>6</v>
@@ -2053,10 +2053,10 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B148" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C148" t="n">
         <v>6</v>
@@ -2064,10 +2064,10 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B149" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C149" t="n">
         <v>4</v>
@@ -2075,10 +2075,10 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B150" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C150" t="n">
         <v>7</v>
@@ -2086,10 +2086,10 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B151" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C151" t="n">
         <v>6</v>
@@ -2097,10 +2097,10 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B152" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C152" t="n">
         <v>7</v>
@@ -2108,10 +2108,10 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B153" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C153" t="n">
         <v>4</v>
@@ -2119,10 +2119,10 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B154" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C154" t="n">
         <v>6</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B155" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C155" t="n">
         <v>6</v>
@@ -2141,10 +2141,10 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B156" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C156" t="n">
         <v>6</v>
@@ -2152,10 +2152,10 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B157" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C157" t="n">
         <v>6</v>
@@ -2163,10 +2163,10 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B158" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C158" t="n">
         <v>5</v>
@@ -2174,10 +2174,10 @@
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B159" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C159" t="n">
         <v>6</v>
@@ -2185,10 +2185,10 @@
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B160" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C160" t="n">
         <v>6</v>
@@ -2196,10 +2196,10 @@
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B161" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C161" t="n">
         <v>4</v>
@@ -2207,10 +2207,10 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B162" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C162" t="n">
         <v>6</v>
@@ -2218,10 +2218,10 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B163" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C163" t="n">
         <v>7</v>
@@ -2229,10 +2229,10 @@
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B164" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C164" t="n">
         <v>4</v>
@@ -2240,10 +2240,10 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B165" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C165" t="n">
         <v>5</v>
@@ -2251,10 +2251,10 @@
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B166" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C166" t="n">
         <v>4</v>
@@ -2262,10 +2262,10 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B167" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C167" t="n">
         <v>3</v>
@@ -2273,10 +2273,10 @@
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B168" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C168" t="n">
         <v>6</v>
@@ -2284,10 +2284,10 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B169" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C169" t="n">
         <v>6</v>
@@ -2295,10 +2295,10 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B170" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C170" t="n">
         <v>6</v>
@@ -2306,10 +2306,10 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B171" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C171" t="n">
         <v>5</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B172" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C172" t="n">
         <v>3</v>
@@ -2328,10 +2328,10 @@
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B173" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C173" t="n">
         <v>5</v>
@@ -2339,10 +2339,10 @@
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B174" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C174" t="n">
         <v>4</v>
@@ -2350,10 +2350,10 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B175" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C175" t="n">
         <v>4</v>
@@ -2361,10 +2361,10 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>4.04</v>
+        <v>3.88</v>
       </c>
       <c r="B176" t="n">
-        <v>8.69</v>
+        <v>10.93</v>
       </c>
       <c r="C176" t="n">
         <v>9</v>
@@ -2372,10 +2372,10 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B177" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C177" t="n">
         <v>6</v>
@@ -2383,10 +2383,10 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B178" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C178" t="n">
         <v>4</v>
@@ -2394,10 +2394,10 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B179" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C179" t="n">
         <v>7</v>
@@ -2405,10 +2405,10 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B180" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C180" t="n">
         <v>4</v>
@@ -2416,10 +2416,10 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B181" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C181" t="n">
         <v>4</v>
@@ -2427,10 +2427,10 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B182" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C182" t="n">
         <v>5</v>
@@ -2441,7 +2441,7 @@
         <v>3.64</v>
       </c>
       <c r="B183" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C183" t="n">
         <v>8</v>
@@ -2449,10 +2449,10 @@
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B184" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C184" t="n">
         <v>6</v>
@@ -2463,7 +2463,7 @@
         <v>3.64</v>
       </c>
       <c r="B185" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C185" t="n">
         <v>8</v>
@@ -2471,10 +2471,10 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B186" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C186" t="n">
         <v>5</v>
@@ -2482,10 +2482,10 @@
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B187" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C187" t="n">
         <v>6</v>
@@ -2493,10 +2493,10 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B188" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C188" t="n">
         <v>6</v>
@@ -2507,7 +2507,7 @@
         <v>3.64</v>
       </c>
       <c r="B189" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C189" t="n">
         <v>8</v>
@@ -2518,7 +2518,7 @@
         <v>3.64</v>
       </c>
       <c r="B190" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C190" t="n">
         <v>8</v>
@@ -2526,10 +2526,10 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B191" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C191" t="n">
         <v>7</v>
@@ -2537,10 +2537,10 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B192" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C192" t="n">
         <v>5</v>
@@ -2548,10 +2548,10 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B193" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C193" t="n">
         <v>5</v>
@@ -2559,10 +2559,10 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B194" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C194" t="n">
         <v>6</v>
@@ -2570,10 +2570,10 @@
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B195" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C195" t="n">
         <v>6</v>
@@ -2581,10 +2581,10 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B196" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C196" t="n">
         <v>5</v>
@@ -2592,10 +2592,10 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B197" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C197" t="n">
         <v>7</v>
@@ -2603,10 +2603,10 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B198" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C198" t="n">
         <v>6</v>
@@ -2614,10 +2614,10 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B199" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C199" t="n">
         <v>6</v>
@@ -2625,10 +2625,10 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B200" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C200" t="n">
         <v>6</v>
@@ -2636,10 +2636,10 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B201" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C201" t="n">
         <v>6</v>
@@ -2647,10 +2647,10 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B202" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C202" t="n">
         <v>6</v>
@@ -2658,10 +2658,10 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B203" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C203" t="n">
         <v>3</v>
@@ -2669,10 +2669,10 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B204" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C204" t="n">
         <v>6</v>
@@ -2680,10 +2680,10 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B205" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C205" t="n">
         <v>5</v>
@@ -2691,10 +2691,10 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B206" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C206" t="n">
         <v>6</v>
@@ -2702,10 +2702,10 @@
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B207" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C207" t="n">
         <v>5</v>
@@ -2713,10 +2713,10 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B208" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C208" t="n">
         <v>6</v>
@@ -2724,10 +2724,10 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B209" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C209" t="n">
         <v>6</v>
@@ -2735,10 +2735,10 @@
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B210" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C210" t="n">
         <v>6</v>
@@ -2746,10 +2746,10 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B211" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C211" t="n">
         <v>6</v>
@@ -2757,10 +2757,10 @@
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B212" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C212" t="n">
         <v>6</v>
@@ -2768,10 +2768,10 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B213" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C213" t="n">
         <v>5</v>
@@ -2779,10 +2779,10 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B214" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C214" t="n">
         <v>4</v>
@@ -2790,10 +2790,10 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B215" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C215" t="n">
         <v>4</v>
@@ -2801,10 +2801,10 @@
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B216" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C216" t="n">
         <v>5</v>
@@ -2812,10 +2812,10 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B217" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C217" t="n">
         <v>4</v>
@@ -2823,10 +2823,10 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B218" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C218" t="n">
         <v>4</v>
@@ -2834,10 +2834,10 @@
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B219" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C219" t="n">
         <v>6</v>
@@ -2845,10 +2845,10 @@
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B220" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C220" t="n">
         <v>5</v>
@@ -2856,10 +2856,10 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B221" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C221" t="n">
         <v>7</v>
@@ -2867,10 +2867,10 @@
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B222" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C222" t="n">
         <v>5</v>
@@ -2878,10 +2878,10 @@
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B223" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C223" t="n">
         <v>4</v>
@@ -2889,10 +2889,10 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="B224" t="n">
-        <v>3.06</v>
+        <v>5.01</v>
       </c>
       <c r="C224" t="n">
         <v>3</v>
@@ -2903,7 +2903,7 @@
         <v>3.64</v>
       </c>
       <c r="B225" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C225" t="n">
         <v>8</v>
@@ -2911,10 +2911,10 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B226" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C226" t="n">
         <v>5</v>
@@ -2922,10 +2922,10 @@
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B227" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C227" t="n">
         <v>5</v>
@@ -2933,10 +2933,10 @@
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B228" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C228" t="n">
         <v>6</v>
@@ -2947,7 +2947,7 @@
         <v>3.64</v>
       </c>
       <c r="B229" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C229" t="n">
         <v>8</v>
@@ -2958,7 +2958,7 @@
         <v>3.64</v>
       </c>
       <c r="B230" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C230" t="n">
         <v>8</v>
@@ -2966,10 +2966,10 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B231" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C231" t="n">
         <v>4</v>
@@ -2977,10 +2977,10 @@
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B232" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C232" t="n">
         <v>6</v>
@@ -2988,10 +2988,10 @@
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B233" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C233" t="n">
         <v>4</v>
@@ -2999,10 +2999,10 @@
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B234" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C234" t="n">
         <v>6</v>
@@ -3010,10 +3010,10 @@
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B235" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C235" t="n">
         <v>6</v>
@@ -3021,10 +3021,10 @@
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B236" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C236" t="n">
         <v>7</v>
@@ -3032,10 +3032,10 @@
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B237" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C237" t="n">
         <v>6</v>
@@ -3046,7 +3046,7 @@
         <v>3.64</v>
       </c>
       <c r="B238" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C238" t="n">
         <v>8</v>
@@ -3054,10 +3054,10 @@
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B239" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C239" t="n">
         <v>6</v>
@@ -3065,10 +3065,10 @@
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B240" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C240" t="n">
         <v>6</v>
@@ -3076,10 +3076,10 @@
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B241" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C241" t="n">
         <v>6</v>
@@ -3087,10 +3087,10 @@
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B242" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C242" t="n">
         <v>5</v>
@@ -3098,10 +3098,10 @@
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B243" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C243" t="n">
         <v>6</v>
@@ -3109,10 +3109,10 @@
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B244" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C244" t="n">
         <v>4</v>
@@ -3123,7 +3123,7 @@
         <v>3.64</v>
       </c>
       <c r="B245" t="n">
-        <v>7.78</v>
+        <v>10.07</v>
       </c>
       <c r="C245" t="n">
         <v>8</v>
@@ -3131,10 +3131,10 @@
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B246" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C246" t="n">
         <v>5</v>
@@ -3142,10 +3142,10 @@
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B247" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C247" t="n">
         <v>5</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B248" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C248" t="n">
         <v>7</v>
@@ -3164,10 +3164,10 @@
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B249" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C249" t="n">
         <v>6</v>
@@ -3175,10 +3175,10 @@
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B250" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C250" t="n">
         <v>4</v>
@@ -3186,10 +3186,10 @@
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B251" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C251" t="n">
         <v>6</v>
@@ -3197,10 +3197,10 @@
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B252" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C252" t="n">
         <v>6</v>
@@ -3208,10 +3208,10 @@
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B253" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C253" t="n">
         <v>4</v>
@@ -3219,10 +3219,10 @@
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>1.95</v>
+        <v>2.47</v>
       </c>
       <c r="B254" t="n">
-        <v>4.03</v>
+        <v>6.15</v>
       </c>
       <c r="C254" t="n">
         <v>4</v>
@@ -3230,10 +3230,10 @@
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>3.22</v>
+        <v>3.37</v>
       </c>
       <c r="B255" t="n">
-        <v>6.84</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="C255" t="n">
         <v>7</v>
@@ -3241,10 +3241,10 @@
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B256" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C256" t="n">
         <v>5</v>
@@ -3252,10 +3252,10 @@
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B257" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C257" t="n">
         <v>5</v>
@@ -3263,10 +3263,10 @@
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B258" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C258" t="n">
         <v>6</v>
@@ -3274,10 +3274,10 @@
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B259" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C259" t="n">
         <v>5</v>
@@ -3285,10 +3285,10 @@
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>4.04</v>
+        <v>3.88</v>
       </c>
       <c r="B260" t="n">
-        <v>8.69</v>
+        <v>10.93</v>
       </c>
       <c r="C260" t="n">
         <v>9</v>
@@ -3296,10 +3296,10 @@
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B261" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C261" t="n">
         <v>5</v>
@@ -3307,10 +3307,10 @@
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B262" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C262" t="n">
         <v>5</v>
@@ -3318,10 +3318,10 @@
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B263" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C263" t="n">
         <v>5</v>
@@ -3329,10 +3329,10 @@
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B264" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C264" t="n">
         <v>5</v>
@@ -3340,10 +3340,10 @@
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B265" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C265" t="n">
         <v>5</v>
@@ -3351,10 +3351,10 @@
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>2.81</v>
+        <v>3.1</v>
       </c>
       <c r="B266" t="n">
-        <v>5.93</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C266" t="n">
         <v>6</v>
@@ -3362,10 +3362,10 @@
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>2.38</v>
+        <v>2.79</v>
       </c>
       <c r="B267" t="n">
-        <v>4.98</v>
+        <v>7.17</v>
       </c>
       <c r="C267" t="n">
         <v>5</v>

</xml_diff>